<commit_message>
Paliers: banque mensuelle de consultations gratuites par tranche de personnes couvertes (code, famille sans abonnement, déduction jusqu'à zéro, non cumulable) — 8 $ inchangé
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T8ao8kQtd2348jDRjtEdaK
</commit_message>
<xml_diff>
--- a/entreprises/registre-modele.xlsx
+++ b/entreprises/registre-modele.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos Faviel Font\truckstopsante-site\entreprises\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368F1DDB-A1E4-4B6C-88EE-AB4D239B2B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF0DC88B-A700-4848-B60C-68E0047C682B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registre" sheetId="1" r:id="rId1"/>
     <sheet name="Facturation" sheetId="2" r:id="rId2"/>
     <sheet name="Instructions" sheetId="3" r:id="rId3"/>
+    <sheet name="Accès gratuits" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
   <si>
     <t>#</t>
   </si>
@@ -261,6 +262,54 @@
   <si>
     <t>FACTURATION MENSUELLE — LA CLINIQUE FACTURE L'ENTREPRISE (les membres ne paient jamais la clinique)</t>
   </si>
+  <si>
+    <t>BANQUE DE CONSULTATIONS GRATUITES - POUR QUI l'entreprise VEUT (pas besoin de payer, envoyez-les-nous)</t>
+  </si>
+  <si>
+    <t>Personnes ACTIVES au registre (en direct) :</t>
+  </si>
+  <si>
+    <t>Règle : 5 consultations gratuites par mois par tranche de 100 personnes couvertes (1 000 = 50)</t>
+  </si>
+  <si>
+    <t>CONSULTATIONS GRATUITES DISPONIBLES CE MOIS :</t>
+  </si>
+  <si>
+    <t>Utilisées ce mois (compte automatique des lignes du mois courant) :</t>
+  </si>
+  <si>
+    <t>Restantes ce mois :</t>
+  </si>
+  <si>
+    <t>Date d'envoi</t>
+  </si>
+  <si>
+    <t>Envoyé par (ARPQ / entreprise)</t>
+  </si>
+  <si>
+    <t>Invité Spruce le</t>
+  </si>
+  <si>
+    <t>Notes (jamais de données de santé)</t>
+  </si>
+  <si>
+    <t>Marc</t>
+  </si>
+  <si>
+    <t>Exemple</t>
+  </si>
+  <si>
+    <t>514 555-0100</t>
+  </si>
+  <si>
+    <t>marc@exemple.com</t>
+  </si>
+  <si>
+    <t>Steve B.</t>
+  </si>
+  <si>
+    <t>EXEMPLE - supprimer cette ligne</t>
+  </si>
 </sst>
 </file>
 
@@ -270,7 +319,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="#,##0\ \$"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -283,74 +332,111 @@
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <i/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF14264A"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -385,6 +471,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF59E0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF14264A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF59E0B"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -422,7 +520,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -460,6 +558,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10563,4 +10667,129 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45FA55C2-8A01-4622-A9B6-8B7BC200582B}">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="60.77734375" customWidth="1"/>
+    <col min="2" max="2" width="14.77734375" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" customWidth="1"/>
+    <col min="5" max="5" width="26.77734375" customWidth="1"/>
+    <col min="6" max="6" width="28.77734375" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" customWidth="1"/>
+    <col min="8" max="8" width="40.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A1" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3">
+        <f>Facturation!B5</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="28">
+        <f>INT(B3/100)*5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6">
+        <f ca="1">COUNTIFS(A10:A509,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),A10:A509,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="27">
+        <f ca="1">B5-B6</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="G9" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="H9" s="29" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="30">
+        <v>46280</v>
+      </c>
+      <c r="B10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" t="s">
+        <v>88</v>
+      </c>
+      <c r="F10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>